<commit_message>
chore: update lead import spreadsheet and remove sample review csv
</commit_message>
<xml_diff>
--- a/import lead.xlsx
+++ b/import lead.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1419" uniqueCount="561">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1472" uniqueCount="578">
   <si>
     <t>category</t>
   </si>
@@ -1694,6 +1694,57 @@
   </si>
   <si>
     <t>mateo.f@example.com</t>
+  </si>
+  <si>
+    <t>500 Ocean Drive</t>
+  </si>
+  <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>Doe</t>
+  </si>
+  <si>
+    <t>(305) 555-1111</t>
+  </si>
+  <si>
+    <t>john.doe@example.com</t>
+  </si>
+  <si>
+    <t>123 Incomplete Way</t>
+  </si>
+  <si>
+    <t>Alex</t>
+  </si>
+  <si>
+    <t>Smith</t>
+  </si>
+  <si>
+    <t>Emma</t>
+  </si>
+  <si>
+    <t>Watson</t>
+  </si>
+  <si>
+    <t>(813) 555-2222</t>
+  </si>
+  <si>
+    <t>emma.w@example.com</t>
+  </si>
+  <si>
+    <t>[link removed]</t>
+  </si>
+  <si>
+    <t>888 Complete Blvd</t>
+  </si>
+  <si>
+    <t>Brown</t>
+  </si>
+  <si>
+    <t>(954) 555-3333</t>
+  </si>
+  <si>
+    <t>michael.b@example.com</t>
   </si>
 </sst>
 </file>
@@ -1744,7 +1795,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1765,6 +1816,21 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8034,6 +8100,236 @@
         <v>52</v>
       </c>
     </row>
+    <row r="102" ht="19.5" customHeight="1">
+      <c r="A102" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B102" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C102" s="7" t="s">
+        <v>561</v>
+      </c>
+      <c r="D102" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="E102" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F102" s="8">
+        <v>33139.0</v>
+      </c>
+      <c r="G102" s="9">
+        <v>750000.0</v>
+      </c>
+      <c r="H102" s="9">
+        <v>210000.0</v>
+      </c>
+      <c r="I102" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="J102" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="K102" s="10">
+        <v>46376.0</v>
+      </c>
+      <c r="L102" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="M102" s="8">
+        <v>5.0</v>
+      </c>
+      <c r="N102" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="O102" s="7" t="s">
+        <v>562</v>
+      </c>
+      <c r="P102" s="7" t="s">
+        <v>563</v>
+      </c>
+      <c r="Q102" s="7" t="s">
+        <v>564</v>
+      </c>
+      <c r="R102" s="7" t="s">
+        <v>565</v>
+      </c>
+      <c r="S102" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="103" ht="19.5" customHeight="1">
+      <c r="A103" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B103" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C103" s="7" t="s">
+        <v>566</v>
+      </c>
+      <c r="D103" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E103" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F103" s="8">
+        <v>32801.0</v>
+      </c>
+      <c r="G103" s="9">
+        <v>420000.0</v>
+      </c>
+      <c r="H103" s="9">
+        <v>110000.0</v>
+      </c>
+      <c r="I103" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="J103" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="K103" s="10">
+        <v>46351.0</v>
+      </c>
+      <c r="L103" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="M103" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="N103" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="O103" s="7" t="s">
+        <v>567</v>
+      </c>
+      <c r="P103" s="7" t="s">
+        <v>568</v>
+      </c>
+      <c r="Q103" s="11"/>
+      <c r="R103" s="11"/>
+      <c r="S103" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="104" ht="19.5" customHeight="1">
+      <c r="A104" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B104" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C104" s="11"/>
+      <c r="D104" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="E104" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F104" s="8">
+        <v>33602.0</v>
+      </c>
+      <c r="G104" s="9">
+        <v>380000.0</v>
+      </c>
+      <c r="H104" s="9">
+        <v>95000.0</v>
+      </c>
+      <c r="I104" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="J104" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="K104" s="10">
+        <v>46397.0</v>
+      </c>
+      <c r="L104" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="M104" s="8">
+        <v>5.0</v>
+      </c>
+      <c r="N104" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="O104" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="P104" s="7" t="s">
+        <v>570</v>
+      </c>
+      <c r="Q104" s="7" t="s">
+        <v>571</v>
+      </c>
+      <c r="R104" s="7" t="s">
+        <v>572</v>
+      </c>
+      <c r="S104" s="7" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="105" ht="19.5" customHeight="1">
+      <c r="A105" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B105" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C105" s="7" t="s">
+        <v>574</v>
+      </c>
+      <c r="D105" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="E105" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F105" s="8">
+        <v>33301.0</v>
+      </c>
+      <c r="G105" s="9">
+        <v>620000.0</v>
+      </c>
+      <c r="H105" s="9">
+        <v>180000.0</v>
+      </c>
+      <c r="I105" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="J105" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="K105" s="10">
+        <v>46402.0</v>
+      </c>
+      <c r="L105" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="M105" s="8">
+        <v>5.0</v>
+      </c>
+      <c r="N105" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="O105" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="P105" s="7" t="s">
+        <v>575</v>
+      </c>
+      <c r="Q105" s="7" t="s">
+        <v>576</v>
+      </c>
+      <c r="R105" s="7" t="s">
+        <v>577</v>
+      </c>
+      <c r="S105" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="S2"/>
@@ -8136,10 +8432,13 @@
     <hyperlink r:id="rId98" ref="S99"/>
     <hyperlink r:id="rId99" ref="S100"/>
     <hyperlink r:id="rId100" ref="S101"/>
+    <hyperlink r:id="rId101" ref="S102"/>
+    <hyperlink r:id="rId102" ref="S103"/>
+    <hyperlink r:id="rId103" ref="S105"/>
   </hyperlinks>
-  <drawing r:id="rId101"/>
+  <drawing r:id="rId104"/>
   <tableParts count="1">
-    <tablePart r:id="rId103"/>
+    <tablePart r:id="rId106"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>